<commit_message>
promote: apply two-column age fields across full 2026 public hunt-table exports
</commit_message>
<xml_diff>
--- a/processed_data/hard_data_exports/hunt_tables/2026/CLEAN_XLXS_STAGED/2026 BISON COW ONLY ONCE-IN-A-LIFETIME ANY LEGAL WEAPON.xlsx
+++ b/processed_data/hard_data_exports/hunt_tables/2026/CLEAN_XLXS_STAGED/2026 BISON COW ONLY ONCE-IN-A-LIFETIME ANY LEGAL WEAPON.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -577,10 +577,15 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Average Age Harvested (previous hunting season)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+          <t>Average Harvest Age</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Current Age (3-Yr Avg)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Avg Days Hunted (previous hunting season)</t>
         </is>
@@ -653,7 +658,8 @@
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -722,7 +728,8 @@
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
@@ -791,7 +798,8 @@
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
@@ -860,7 +868,8 @@
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr"/>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
@@ -921,7 +930,8 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O6"/>

</xml_diff>